<commit_message>
fix: remove large number test case
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/TRIGONOMETRIC.xlsx
+++ b/xlsx/tests/calc_tests/MATH_AND_TRIGONOMETRY/TRIGONOMETRIC.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7894C87D-E032-44C0-AA5F-F73E0B8A2FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82358F3-ABBC-496E-92B8-42A5E28C132B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5090" yWindow="2450" windowWidth="27470" windowHeight="16370" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SIN_COS_TAN" sheetId="10" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="55">
   <si>
     <t>Number</t>
   </si>
@@ -267,7 +267,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,12 +277,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -314,7 +308,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -328,9 +322,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -635,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC33E34-CC5A-470E-A24C-36B3C446A422}">
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr defaultColWidth="14.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.6328125" customWidth="1"/>
@@ -988,49 +979,46 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="5">
-        <v>9999999999999</v>
-      </c>
-      <c r="B20" s="9" t="e">
+      <c r="A20" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" s="6">
         <f>SIN(A20)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="C20" s="9" t="e">
+        <v>0.8414709848078965</v>
+      </c>
+      <c r="C20" s="6">
         <f>COS(A20)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="D20" s="9" t="e">
+        <v>0.54030230586813977</v>
+      </c>
+      <c r="D20" s="6">
         <f>TAN(A20)</f>
-        <v>#NUM!</v>
+        <v>1.5574077246549023</v>
       </c>
       <c r="E20" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" s="6">
         <f>SIN(A21)</f>
-        <v>0.8414709848078965</v>
+        <v>0</v>
       </c>
       <c r="C21" s="6">
         <f>COS(A21)</f>
-        <v>0.54030230586813977</v>
+        <v>1</v>
       </c>
       <c r="D21" s="6">
         <f>TAN(A21)</f>
-        <v>1.5574077246549023</v>
+        <v>0</v>
       </c>
       <c r="E21" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="b">
-        <v>0</v>
-      </c>
       <c r="B22" s="6">
         <f>SIN(A22)</f>
         <v>0</v>
@@ -1044,83 +1032,87 @@
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B23" s="6">
+      <c r="A23" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="B23" s="6" t="e">
         <f>SIN(A23)</f>
-        <v>0</v>
-      </c>
-      <c r="C23" s="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C23" s="6" t="e">
         <f>COS(A23)</f>
-        <v>1</v>
-      </c>
-      <c r="D23" s="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D23" s="6" t="e">
         <f>TAN(A23)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E23" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="str">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="B24" s="6" t="e">
-        <f>SIN(A24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C24" s="6" t="e">
-        <f>COS(A24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D24" s="6" t="e">
-        <f>TAN(A24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E24" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" t="str">
         <f>"8"</f>
         <v>8</v>
       </c>
+      <c r="B24" s="6">
+        <f>SIN(A24)</f>
+        <v>0.98935824662338179</v>
+      </c>
+      <c r="C24" s="6">
+        <f>COS(A24)</f>
+        <v>-0.14550003380861354</v>
+      </c>
+      <c r="D24" s="6">
+        <f>TAN(A24)</f>
+        <v>-6.799711455220379</v>
+      </c>
+      <c r="E24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>2</v>
+      </c>
       <c r="B25" s="6">
         <f>SIN(A25)</f>
-        <v>0.98935824662338179</v>
+        <v>0.90929742682568171</v>
       </c>
       <c r="C25" s="6">
         <f>COS(A25)</f>
-        <v>-0.14550003380861354</v>
+        <v>-0.41614683654714241</v>
       </c>
       <c r="D25" s="6">
         <f>TAN(A25)</f>
-        <v>-6.799711455220379</v>
+        <v>-2.1850398632615189</v>
       </c>
       <c r="E25" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>2</v>
+      <c r="A26" t="str">
+        <f>" 10 "</f>
+        <v xml:space="preserve"> 10 </v>
       </c>
       <c r="B26" s="6">
         <f>SIN(A26)</f>
-        <v>0.90929742682568171</v>
+        <v>-0.54402111088936977</v>
       </c>
       <c r="C26" s="6">
         <f>COS(A26)</f>
-        <v>-0.41614683654714241</v>
+        <v>-0.83907152907645244</v>
       </c>
       <c r="D26" s="6">
         <f>TAN(A26)</f>
-        <v>-2.1850398632615189</v>
+        <v>0.64836082745908663</v>
       </c>
       <c r="E26" t="s">
         <v>7</v>
@@ -1128,124 +1120,124 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="str">
-        <f>" 10 "</f>
-        <v xml:space="preserve"> 10 </v>
+        <f>"0"</f>
+        <v>0</v>
       </c>
       <c r="B27" s="6">
         <f>SIN(A27)</f>
-        <v>-0.54402111088936977</v>
+        <v>0</v>
       </c>
       <c r="C27" s="6">
         <f>COS(A27)</f>
-        <v>-0.83907152907645244</v>
+        <v>1</v>
       </c>
       <c r="D27" s="6">
         <f>TAN(A27)</f>
-        <v>0.64836082745908663</v>
+        <v>0</v>
       </c>
       <c r="E27" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" t="str">
-        <f>"0"</f>
-        <v>0</v>
-      </c>
-      <c r="B28" s="6">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" s="6" t="e">
         <f>SIN(A28)</f>
-        <v>0</v>
-      </c>
-      <c r="C28" s="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C28" s="6" t="e">
         <f>COS(A28)</f>
-        <v>1</v>
-      </c>
-      <c r="D28" s="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D28" s="6" t="e">
         <f>TAN(A28)</f>
-        <v>0</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E28" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>8</v>
+      <c r="A29" s="2" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="B29" s="6" t="e">
         <f>SIN(A29)</f>
-        <v>#VALUE!</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C29" s="6" t="e">
         <f>COS(A29)</f>
-        <v>#VALUE!</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D29" s="6" t="e">
         <f>TAN(A29)</f>
-        <v>#VALUE!</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="E29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="e">
-        <f>1/0</f>
-        <v>#DIV/0!</v>
+      <c r="A30" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
       </c>
       <c r="B30" s="6" t="e">
         <f>SIN(A30)</f>
-        <v>#DIV/0!</v>
+        <v>#N/A</v>
       </c>
       <c r="C30" s="6" t="e">
         <f>COS(A30)</f>
-        <v>#DIV/0!</v>
+        <v>#N/A</v>
       </c>
       <c r="D30" s="6" t="e">
         <f>TAN(A30)</f>
-        <v>#DIV/0!</v>
+        <v>#N/A</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+      <c r="A31" t="e" cm="1">
+        <f t="array" ref="A31">HELLO</f>
+        <v>#NAME?</v>
       </c>
       <c r="B31" s="6" t="e">
         <f>SIN(A31)</f>
-        <v>#N/A</v>
+        <v>#NAME?</v>
       </c>
       <c r="C31" s="6" t="e">
         <f>COS(A31)</f>
-        <v>#N/A</v>
+        <v>#NAME?</v>
       </c>
       <c r="D31" s="6" t="e">
         <f>TAN(A31)</f>
-        <v>#N/A</v>
+        <v>#NAME?</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" t="e" cm="1">
-        <f t="array" ref="A32">HELLO</f>
-        <v>#NAME?</v>
+      <c r="A32" t="e">
+        <f>SQRT(-1)</f>
+        <v>#NUM!</v>
       </c>
       <c r="B32" s="6" t="e">
         <f>SIN(A32)</f>
-        <v>#NAME?</v>
+        <v>#NUM!</v>
       </c>
       <c r="C32" s="6" t="e">
         <f>COS(A32)</f>
-        <v>#NAME?</v>
+        <v>#NUM!</v>
       </c>
       <c r="D32" s="6" t="e">
         <f>TAN(A32)</f>
-        <v>#NAME?</v>
+        <v>#NUM!</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -1253,92 +1245,95 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="e">
-        <f>SQRT(-1)</f>
-        <v>#NUM!</v>
+        <f>"x"+1</f>
+        <v>#VALUE!</v>
       </c>
       <c r="B33" s="6" t="e">
         <f>SIN(A33)</f>
-        <v>#NUM!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C33" s="6" t="e">
         <f>COS(A33)</f>
-        <v>#NUM!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="D33" s="6" t="e">
         <f>TAN(A33)</f>
-        <v>#NUM!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" t="e">
-        <f>"x"+1</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B34" s="6" t="e">
-        <f>SIN(A34)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C34" s="6" t="e">
-        <f>COS(A34)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D34" s="6" t="e">
-        <f>TAN(A34)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E34" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35">
+      <c r="A34">
         <f>2^20</f>
         <v>1048576</v>
       </c>
-      <c r="B35" s="6">
-        <f>SIN(A35)</f>
+      <c r="B34" s="6">
+        <f>SIN(A34)</f>
         <v>0.33049314002171887</v>
       </c>
-      <c r="C35" s="6">
-        <f>COS(A35)</f>
+      <c r="C34" s="6">
+        <f>COS(A34)</f>
         <v>0.94380839390131754</v>
       </c>
-      <c r="D35" s="6">
-        <f>TAN(A35)</f>
+      <c r="D34" s="6">
+        <f>TAN(A34)</f>
         <v>0.35016974012659025</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E34" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A36" t="str">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" t="str">
         <f>"@"</f>
         <v>@</v>
       </c>
-      <c r="B36" s="6" t="e">
-        <f>SIN(A36)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C36" s="6" t="e">
-        <f>COS(A36)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D36" s="6" t="e">
-        <f>TAN(A36)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E36" t="s">
+      <c r="B35" s="6" t="e">
+        <f>SIN(A35)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C35" s="6" t="e">
+        <f>COS(A35)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D35" s="6" t="e">
+        <f>TAN(A35)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E35" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A37" s="2">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
         <f>DATE(2024,1,10)</f>
         <v>45301</v>
+      </c>
+      <c r="B36" s="6">
+        <f>SIN(A36)</f>
+        <v>-0.69330470840023772</v>
+      </c>
+      <c r="C36" s="6">
+        <f>COS(A36)</f>
+        <v>0.72064455962010932</v>
+      </c>
+      <c r="D36" s="6">
+        <f>TAN(A36)</f>
+        <v>-0.96206194738459705</v>
+      </c>
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="I36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" t="str">
+        <f>"2024-01-10"</f>
+        <v>2024-01-10</v>
       </c>
       <c r="B37" s="6">
         <f>SIN(A37)</f>
@@ -1353,197 +1348,194 @@
         <v>-0.96206194738459705</v>
       </c>
       <c r="E37" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="str">
-        <f>"2024-01-10"</f>
-        <v>2024-01-10</v>
-      </c>
-      <c r="B38" s="6">
-        <f>SIN(A38)</f>
-        <v>-0.69330470840023772</v>
-      </c>
-      <c r="C38" s="6">
-        <f>COS(A38)</f>
-        <v>0.72064455962010932</v>
-      </c>
-      <c r="D38" s="6">
-        <f>TAN(A38)</f>
-        <v>-0.96206194738459705</v>
-      </c>
-      <c r="E38" t="s">
-        <v>14</v>
-      </c>
-      <c r="I38">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A39" t="str">
         <f>" 2024-01-10 "</f>
         <v xml:space="preserve"> 2024-01-10 </v>
       </c>
-      <c r="B39" s="6" t="e">
-        <f>SIN(A39)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C39" s="6" t="e">
-        <f>COS(A39)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D39" s="6" t="e">
-        <f>TAN(A39)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E39" t="s">
+      <c r="B38" s="6" t="e">
+        <f>SIN(A38)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C38" s="6" t="e">
+        <f>COS(A38)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D38" s="6" t="e">
+        <f>TAN(A38)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E38" t="s">
         <v>15</v>
       </c>
-      <c r="I39">
+      <c r="I38">
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A40" s="4">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="4">
         <f>TIME(14,30,0)</f>
         <v>0.60416666666666663</v>
       </c>
+      <c r="B39" s="6">
+        <f>SIN(A39)</f>
+        <v>0.56807646043671656</v>
+      </c>
+      <c r="C39" s="6">
+        <f>COS(A39)</f>
+        <v>0.82297578038341535</v>
+      </c>
+      <c r="D39" s="6">
+        <f>TAN(A39)</f>
+        <v>0.69027117684077655</v>
+      </c>
+      <c r="E39" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B40" s="6">
-        <f>SIN(A40)</f>
-        <v>0.56807646043671656</v>
-      </c>
-      <c r="C40" s="6">
-        <f>COS(A40)</f>
-        <v>0.82297578038341535</v>
-      </c>
-      <c r="D40" s="6">
-        <f>TAN(A40)</f>
-        <v>0.69027117684077655</v>
-      </c>
-      <c r="E40" t="s">
-        <v>16</v>
-      </c>
-      <c r="I40">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B41" s="6">
         <f>SIN(I:I)</f>
         <v>-0.95892427466313845</v>
       </c>
-      <c r="C41" s="6">
+      <c r="C40" s="6">
         <f>COS(I:I)</f>
         <v>0.28366218546322625</v>
       </c>
-      <c r="D41" s="6">
+      <c r="D40" s="6">
         <f>TAN(I:I)</f>
         <v>-3.3805150062465859</v>
       </c>
+      <c r="E40" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <f>1.05*(0.0284+0.0046)-0.0284</f>
+        <v>6.2499999999999986E-3</v>
+      </c>
+      <c r="B41" s="6">
+        <f>SIN(A41)</f>
+        <v>6.2499593099753043E-3</v>
+      </c>
+      <c r="C41" s="6">
+        <f>COS(A41)</f>
+        <v>0.99998046881357816</v>
+      </c>
+      <c r="D41" s="6">
+        <f>TAN(A41)</f>
+        <v>6.2500813814799182E-3</v>
+      </c>
       <c r="E41" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I41">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42">
-        <f>1.05*(0.0284+0.0046)-0.0284</f>
-        <v>6.2499999999999986E-3</v>
+        <f>I43</f>
+        <v>1.75</v>
       </c>
       <c r="B42" s="6">
         <f>SIN(A42)</f>
-        <v>6.2499593099753043E-3</v>
+        <v>0.98398594687393692</v>
       </c>
       <c r="C42" s="6">
         <f>COS(A42)</f>
-        <v>0.99998046881357816</v>
+        <v>-0.17824605564949209</v>
       </c>
       <c r="D42" s="6">
         <f>TAN(A42)</f>
-        <v>6.2500813814799182E-3</v>
+        <v>-5.5203799225093304</v>
       </c>
       <c r="E42" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I42">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43">
-        <f>I44</f>
+      <c r="A43" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="6" t="e">
+        <f>SIN(A43)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C43" s="6" t="e">
+        <f>COS(A43)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D43" s="6" t="e">
+        <f>TAN(A43)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I43">
         <v>1.75</v>
       </c>
-      <c r="B43" s="6">
-        <f>SIN(A43)</f>
-        <v>0.98398594687393692</v>
-      </c>
-      <c r="C43" s="6">
-        <f>COS(A43)</f>
-        <v>-0.17824605564949209</v>
-      </c>
-      <c r="D43" s="6">
-        <f>TAN(A43)</f>
-        <v>-5.5203799225093304</v>
-      </c>
-      <c r="E43" t="s">
-        <v>19</v>
-      </c>
-      <c r="I43">
-        <v>7</v>
-      </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>20</v>
-      </c>
-      <c r="B44" s="6" t="e">
+      <c r="A44">
+        <f>PI() - 0.000000000001</f>
+        <v>3.141592653588793</v>
+      </c>
+      <c r="B44" s="7">
         <f>SIN(A44)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C44" s="6" t="e">
+        <v>1.0002114154278319E-12</v>
+      </c>
+      <c r="C44" s="6">
         <f>COS(A44)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D44" s="6" t="e">
+        <v>-1</v>
+      </c>
+      <c r="D44" s="7">
         <f>TAN(A44)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I44">
-        <v>1.75</v>
+        <v>-1.0002114154278319E-12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45">
-        <f>PI() - 0.000000000001</f>
-        <v>3.141592653588793</v>
-      </c>
-      <c r="B45" s="7">
+        <f>PI()/2 - 0.000000000001</f>
+        <v>1.5707963267938965</v>
+      </c>
+      <c r="B45" s="6">
         <f>SIN(A45)</f>
-        <v>1.0002114154278319E-12</v>
-      </c>
-      <c r="C45" s="6">
+        <v>1</v>
+      </c>
+      <c r="C45" s="7">
         <f>COS(A45)</f>
-        <v>-1</v>
+        <v>1.0001501580050864E-12</v>
       </c>
       <c r="D45" s="7">
         <f>TAN(A45)</f>
-        <v>-1.0002114154278319E-12</v>
+        <v>999849864538.95483</v>
       </c>
       <c r="E45" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46">
-        <f>PI()/2 - 0.000000000001</f>
-        <v>1.5707963267938965</v>
+        <f>PI()/2 + 0.000000000001</f>
+        <v>1.5707963267958966</v>
       </c>
       <c r="B46" s="6">
         <f>SIN(A46)</f>
@@ -1551,136 +1543,115 @@
       </c>
       <c r="C46" s="7">
         <f>COS(A46)</f>
-        <v>1.0001501580050864E-12</v>
+        <v>-1.0000276431595956E-12</v>
       </c>
       <c r="D46" s="7">
         <f>TAN(A46)</f>
-        <v>999849864538.95483</v>
+        <v>-999972357604.52759</v>
       </c>
       <c r="E46" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A47">
-        <f>PI()/2 + 0.000000000001</f>
-        <v>1.5707963267958966</v>
-      </c>
-      <c r="B47" s="6">
+      <c r="A47" s="9">
+        <f>PI()</f>
+        <v>3.1415926535897931</v>
+      </c>
+      <c r="B47" s="7">
         <f>SIN(A47)</f>
-        <v>1</v>
-      </c>
-      <c r="C47" s="7">
+        <v>1.22514845490862E-16</v>
+      </c>
+      <c r="C47" s="6">
         <f>COS(A47)</f>
-        <v>-1.0000276431595956E-12</v>
+        <v>-1</v>
       </c>
       <c r="D47" s="7">
         <f>TAN(A47)</f>
-        <v>-999972357604.52759</v>
+        <v>-1.22514845490862E-16</v>
       </c>
       <c r="E47" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="10">
-        <f>PI()</f>
-        <v>3.1415926535897931</v>
-      </c>
-      <c r="B48" s="7">
-        <f>SIN(A48)</f>
-        <v>1.22514845490862E-16</v>
-      </c>
-      <c r="C48" s="6">
-        <f>COS(A48)</f>
-        <v>-1</v>
-      </c>
-      <c r="D48" s="7">
-        <f>TAN(A48)</f>
-        <v>-1.22514845490862E-16</v>
-      </c>
-      <c r="E48" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="10">
+      <c r="A48" s="9">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
-      <c r="B49" s="6">
-        <f>SIN(A49)</f>
+      <c r="B48" s="6">
+        <f>SIN(A48)</f>
         <v>1</v>
       </c>
-      <c r="C49" s="7">
-        <f>COS(A49)</f>
+      <c r="C48" s="7">
+        <f>COS(A48)</f>
         <v>6.1257422745431001E-17</v>
       </c>
-      <c r="D49" s="7"/>
-      <c r="E49" t="s">
+      <c r="D48" s="7"/>
+      <c r="E48" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="10">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="9">
         <f>2*PI()</f>
         <v>6.2831853071795862</v>
       </c>
-      <c r="B50" s="7">
+      <c r="B49" s="7">
+        <f>SIN(A49)</f>
+        <v>-2.45029690981724E-16</v>
+      </c>
+      <c r="C49" s="6">
+        <f>COS(A49)</f>
+        <v>1</v>
+      </c>
+      <c r="D49" s="7">
+        <f>TAN(A49)</f>
+        <v>-2.45029690981724E-16</v>
+      </c>
+      <c r="E49" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="9">
+        <f>PI()/4</f>
+        <v>0.78539816339744828</v>
+      </c>
+      <c r="B50" s="6">
         <f>SIN(A50)</f>
-        <v>-2.45029690981724E-16</v>
+        <v>0.70710678118654746</v>
       </c>
       <c r="C50" s="6">
         <f>COS(A50)</f>
-        <v>1</v>
-      </c>
-      <c r="D50" s="7">
+        <v>0.70710678118654757</v>
+      </c>
+      <c r="D50" s="6">
         <f>TAN(A50)</f>
-        <v>-2.45029690981724E-16</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="E50" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="10">
-        <f>PI()/4</f>
-        <v>0.78539816339744828</v>
+      <c r="A51" s="9">
+        <f>PI()/6</f>
+        <v>0.52359877559829882</v>
       </c>
       <c r="B51" s="6">
         <f>SIN(A51)</f>
-        <v>0.70710678118654746</v>
+        <v>0.49999999999999994</v>
       </c>
       <c r="C51" s="6">
         <f>COS(A51)</f>
-        <v>0.70710678118654757</v>
+        <v>0.86602540378443871</v>
       </c>
       <c r="D51" s="6">
         <f>TAN(A51)</f>
-        <v>0.99999999999999989</v>
+        <v>0.57735026918962573</v>
       </c>
       <c r="E51" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="10">
-        <f>PI()/6</f>
-        <v>0.52359877559829882</v>
-      </c>
-      <c r="B52" s="6">
-        <f>SIN(A52)</f>
-        <v>0.49999999999999994</v>
-      </c>
-      <c r="C52" s="6">
-        <f>COS(A52)</f>
-        <v>0.86602540378443871</v>
-      </c>
-      <c r="D52" s="6">
-        <f>TAN(A52)</f>
-        <v>0.57735026918962573</v>
-      </c>
-      <c r="E52" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2639,7 +2610,7 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="10">
+      <c r="A48" s="9">
         <f>PI()</f>
         <v>3.1415926535897931</v>
       </c>
@@ -2660,7 +2631,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="10">
+      <c r="A49" s="9">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
@@ -2681,7 +2652,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="10">
+      <c r="A50" s="9">
         <f>2*PI()</f>
         <v>6.2831853071795862</v>
       </c>
@@ -2702,7 +2673,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="10">
+      <c r="A51" s="9">
         <f>PI()/4</f>
         <v>0.78539816339744828</v>
       </c>
@@ -2723,7 +2694,7 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="10">
+      <c r="A52" s="9">
         <f>PI()/6</f>
         <v>0.52359877559829882</v>
       </c>
@@ -3698,7 +3669,7 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="10">
+      <c r="A48" s="9">
         <f>PI()</f>
         <v>3.1415926535897931</v>
       </c>
@@ -3719,7 +3690,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="10">
+      <c r="A49" s="9">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
@@ -3740,7 +3711,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="10">
+      <c r="A50" s="9">
         <f>2*PI()</f>
         <v>6.2831853071795862</v>
       </c>
@@ -3761,7 +3732,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="10">
+      <c r="A51" s="9">
         <f>PI()/4</f>
         <v>0.78539816339744828</v>
       </c>
@@ -3782,7 +3753,7 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="10">
+      <c r="A52" s="9">
         <f>PI()/6</f>
         <v>0.52359877559829882</v>
       </c>
@@ -4757,7 +4728,7 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="10">
+      <c r="A48" s="9">
         <f>PI()</f>
         <v>3.1415926535897931</v>
       </c>
@@ -4778,7 +4749,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="10">
+      <c r="A49" s="9">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
@@ -4799,7 +4770,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="10">
+      <c r="A50" s="9">
         <f>2*PI()</f>
         <v>6.2831853071795862</v>
       </c>
@@ -4820,7 +4791,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="10">
+      <c r="A51" s="9">
         <f>PI()/4</f>
         <v>0.78539816339744828</v>
       </c>
@@ -4841,7 +4812,7 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="10">
+      <c r="A52" s="9">
         <f>PI()/6</f>
         <v>0.52359877559829882</v>
       </c>
@@ -4868,7 +4839,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6566592-A507-4EE7-A267-75E161C79488}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultColWidth="14.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="4" width="18" customWidth="1"/>
@@ -5220,49 +5191,46 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="5">
-        <v>9999999999999</v>
-      </c>
-      <c r="B20" s="9" t="e">
+      <c r="A20" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" s="6">
         <f>_xlfn.COT(A20)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="C20" s="9" t="e">
+        <v>0.64209261593433065</v>
+      </c>
+      <c r="C20" s="6">
         <f>_xlfn.CSC(A20)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="D20" s="9" t="e">
+        <v>1.1883951057781212</v>
+      </c>
+      <c r="D20" s="6">
         <f>_xlfn.SEC(A20)</f>
-        <v>#NUM!</v>
+        <v>1.8508157176809255</v>
       </c>
       <c r="E20" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="B21" s="6">
+        <v>0</v>
+      </c>
+      <c r="B21" s="6" t="e">
         <f>_xlfn.COT(A21)</f>
-        <v>0.64209261593433065</v>
-      </c>
-      <c r="C21" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C21" s="6" t="e">
         <f>_xlfn.CSC(A21)</f>
-        <v>1.1883951057781212</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D21" s="6">
         <f>_xlfn.SEC(A21)</f>
-        <v>1.8508157176809255</v>
+        <v>1</v>
       </c>
       <c r="E21" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="b">
-        <v>0</v>
-      </c>
       <c r="B22" s="6" t="e">
         <f>_xlfn.COT(A22)</f>
         <v>#DIV/0!</v>
@@ -5276,83 +5244,87 @@
         <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="str">
+        <f>""</f>
+        <v/>
+      </c>
       <c r="B23" s="6" t="e">
         <f>_xlfn.COT(A23)</f>
-        <v>#DIV/0!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C23" s="6" t="e">
         <f>_xlfn.CSC(A23)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D23" s="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D23" s="6" t="e">
         <f>_xlfn.SEC(A23)</f>
-        <v>1</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E23" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="str">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="B24" s="6" t="e">
-        <f>_xlfn.COT(A24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C24" s="6" t="e">
-        <f>_xlfn.CSC(A24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D24" s="6" t="e">
-        <f>_xlfn.SEC(A24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E24" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" t="str">
         <f>"8"</f>
         <v>8</v>
       </c>
+      <c r="B24" s="6">
+        <f>_xlfn.COT(A24)</f>
+        <v>-0.14706506394948049</v>
+      </c>
+      <c r="C24" s="6">
+        <f>_xlfn.CSC(A24)</f>
+        <v>1.0107562184000971</v>
+      </c>
+      <c r="D24" s="6">
+        <f>_xlfn.SEC(A24)</f>
+        <v>-6.8728506366903703</v>
+      </c>
+      <c r="E24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>2</v>
+      </c>
       <c r="B25" s="6">
         <f>_xlfn.COT(A25)</f>
-        <v>-0.14706506394948049</v>
+        <v>-0.45765755436028577</v>
       </c>
       <c r="C25" s="6">
         <f>_xlfn.CSC(A25)</f>
-        <v>1.0107562184000971</v>
+        <v>1.0997501702946164</v>
       </c>
       <c r="D25" s="6">
         <f>_xlfn.SEC(A25)</f>
-        <v>-6.8728506366903703</v>
+        <v>-2.4029979617223809</v>
       </c>
       <c r="E25" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>2</v>
+      <c r="A26" t="str">
+        <f>" 10 "</f>
+        <v xml:space="preserve"> 10 </v>
       </c>
       <c r="B26" s="6">
         <f>_xlfn.COT(A26)</f>
-        <v>-0.45765755436028577</v>
+        <v>1.5423510453569202</v>
       </c>
       <c r="C26" s="6">
         <f>_xlfn.CSC(A26)</f>
-        <v>1.0997501702946164</v>
+        <v>-1.8381639608896658</v>
       </c>
       <c r="D26" s="6">
         <f>_xlfn.SEC(A26)</f>
-        <v>-2.4029979617223809</v>
+        <v>-1.1917935066878957</v>
       </c>
       <c r="E26" t="s">
         <v>7</v>
@@ -5360,124 +5332,124 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="str">
-        <f>" 10 "</f>
-        <v xml:space="preserve"> 10 </v>
-      </c>
-      <c r="B27" s="6">
+        <f>"0"</f>
+        <v>0</v>
+      </c>
+      <c r="B27" s="6" t="e">
         <f>_xlfn.COT(A27)</f>
-        <v>1.5423510453569202</v>
-      </c>
-      <c r="C27" s="6">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C27" s="6" t="e">
         <f>_xlfn.CSC(A27)</f>
-        <v>-1.8381639608896658</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D27" s="6">
         <f>_xlfn.SEC(A27)</f>
-        <v>-1.1917935066878957</v>
+        <v>1</v>
       </c>
       <c r="E27" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" t="str">
-        <f>"0"</f>
-        <v>0</v>
+      <c r="A28" t="s">
+        <v>8</v>
       </c>
       <c r="B28" s="6" t="e">
         <f>_xlfn.COT(A28)</f>
-        <v>#DIV/0!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C28" s="6" t="e">
         <f>_xlfn.CSC(A28)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D28" s="6" t="e">
+        <f>_xlfn.SEC(A28)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="e">
+        <f>1/0</f>
         <v>#DIV/0!</v>
-      </c>
-      <c r="D28" s="6">
-        <f>_xlfn.SEC(A28)</f>
-        <v>1</v>
-      </c>
-      <c r="E28" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>8</v>
       </c>
       <c r="B29" s="6" t="e">
         <f>_xlfn.COT(A29)</f>
-        <v>#VALUE!</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="C29" s="6" t="e">
         <f>_xlfn.CSC(A29)</f>
-        <v>#VALUE!</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="D29" s="6" t="e">
         <f>_xlfn.SEC(A29)</f>
-        <v>#VALUE!</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="E29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="2" t="e">
-        <f>1/0</f>
-        <v>#DIV/0!</v>
+      <c r="A30" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
       </c>
       <c r="B30" s="6" t="e">
         <f>_xlfn.COT(A30)</f>
-        <v>#DIV/0!</v>
+        <v>#N/A</v>
       </c>
       <c r="C30" s="6" t="e">
         <f>_xlfn.CSC(A30)</f>
-        <v>#DIV/0!</v>
+        <v>#N/A</v>
       </c>
       <c r="D30" s="6" t="e">
         <f>_xlfn.SEC(A30)</f>
-        <v>#DIV/0!</v>
+        <v>#N/A</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+      <c r="A31" t="e" cm="1">
+        <f t="array" ref="A31">HELLO</f>
+        <v>#NAME?</v>
       </c>
       <c r="B31" s="6" t="e">
         <f>_xlfn.COT(A31)</f>
-        <v>#N/A</v>
+        <v>#NAME?</v>
       </c>
       <c r="C31" s="6" t="e">
         <f>_xlfn.CSC(A31)</f>
-        <v>#N/A</v>
+        <v>#NAME?</v>
       </c>
       <c r="D31" s="6" t="e">
         <f>_xlfn.SEC(A31)</f>
-        <v>#N/A</v>
+        <v>#NAME?</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" t="e" cm="1">
-        <f t="array" ref="A32">HELLO</f>
-        <v>#NAME?</v>
+      <c r="A32" t="e">
+        <f>SQRT(-1)</f>
+        <v>#NUM!</v>
       </c>
       <c r="B32" s="6" t="e">
         <f>_xlfn.COT(A32)</f>
-        <v>#NAME?</v>
+        <v>#NUM!</v>
       </c>
       <c r="C32" s="6" t="e">
         <f>_xlfn.CSC(A32)</f>
-        <v>#NAME?</v>
+        <v>#NUM!</v>
       </c>
       <c r="D32" s="6" t="e">
         <f>_xlfn.SEC(A32)</f>
-        <v>#NAME?</v>
+        <v>#NUM!</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -5485,92 +5457,95 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="e">
-        <f>SQRT(-1)</f>
-        <v>#NUM!</v>
+        <f>"x"+1</f>
+        <v>#VALUE!</v>
       </c>
       <c r="B33" s="6" t="e">
         <f>_xlfn.COT(A33)</f>
-        <v>#NUM!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="C33" s="6" t="e">
         <f>_xlfn.CSC(A33)</f>
-        <v>#NUM!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="D33" s="6" t="e">
         <f>_xlfn.SEC(A33)</f>
-        <v>#NUM!</v>
+        <v>#VALUE!</v>
       </c>
       <c r="E33" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" t="e">
-        <f>"x"+1</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B34" s="6" t="e">
-        <f>_xlfn.COT(A34)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C34" s="6" t="e">
-        <f>_xlfn.CSC(A34)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D34" s="6" t="e">
-        <f>_xlfn.SEC(A34)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E34" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35">
+      <c r="A34">
         <f>2^20</f>
         <v>1048576</v>
       </c>
-      <c r="B35" s="6">
-        <f>_xlfn.COT(A35)</f>
+      <c r="B34" s="6">
+        <f>_xlfn.COT(A34)</f>
         <v>2.855757895123916</v>
       </c>
-      <c r="C35" s="6">
-        <f>_xlfn.CSC(A35)</f>
+      <c r="C34" s="6">
+        <f>_xlfn.CSC(A34)</f>
         <v>3.0257814123896294</v>
       </c>
-      <c r="D35" s="6">
-        <f>_xlfn.SEC(A35)</f>
+      <c r="D34" s="6">
+        <f>_xlfn.SEC(A34)</f>
         <v>1.0595370908563435</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E34" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A36" t="str">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" t="str">
         <f>"@"</f>
         <v>@</v>
       </c>
-      <c r="B36" s="6" t="e">
-        <f>_xlfn.COT(A36)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C36" s="6" t="e">
-        <f>_xlfn.CSC(A36)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D36" s="6" t="e">
-        <f>_xlfn.SEC(A36)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E36" t="s">
+      <c r="B35" s="6" t="e">
+        <f>_xlfn.COT(A35)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C35" s="6" t="e">
+        <f>_xlfn.CSC(A35)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D35" s="6" t="e">
+        <f>_xlfn.SEC(A35)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E35" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A37" s="2">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
         <f>DATE(2024,1,10)</f>
         <v>45301</v>
+      </c>
+      <c r="B36" s="6">
+        <f>_xlfn.COT(A36)</f>
+        <v>-1.0394341057959304</v>
+      </c>
+      <c r="C36" s="6">
+        <f>_xlfn.CSC(A36)</f>
+        <v>-1.4423672418256681</v>
+      </c>
+      <c r="D36" s="6">
+        <f>_xlfn.SEC(A36)</f>
+        <v>1.3876466375145522</v>
+      </c>
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="I36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" t="str">
+        <f>"2024-01-10"</f>
+        <v>2024-01-10</v>
       </c>
       <c r="B37" s="6">
         <f>_xlfn.COT(A37)</f>
@@ -5585,201 +5560,198 @@
         <v>1.3876466375145522</v>
       </c>
       <c r="E37" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="str">
-        <f>"2024-01-10"</f>
-        <v>2024-01-10</v>
-      </c>
-      <c r="B38" s="6">
-        <f>_xlfn.COT(A38)</f>
-        <v>-1.0394341057959304</v>
-      </c>
-      <c r="C38" s="6">
-        <f>_xlfn.CSC(A38)</f>
-        <v>-1.4423672418256681</v>
-      </c>
-      <c r="D38" s="6">
-        <f>_xlfn.SEC(A38)</f>
-        <v>1.3876466375145522</v>
-      </c>
-      <c r="E38" t="s">
-        <v>14</v>
-      </c>
-      <c r="I38">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A39" t="str">
         <f>" 2024-01-10 "</f>
         <v xml:space="preserve"> 2024-01-10 </v>
       </c>
-      <c r="B39" s="6" t="e">
-        <f>_xlfn.COT(A39)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C39" s="6" t="e">
-        <f>_xlfn.CSC(A39)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D39" s="6" t="e">
-        <f>_xlfn.SEC(A39)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E39" t="s">
+      <c r="B38" s="6" t="e">
+        <f>_xlfn.COT(A38)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C38" s="6" t="e">
+        <f>_xlfn.CSC(A38)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D38" s="6" t="e">
+        <f>_xlfn.SEC(A38)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E38" t="s">
         <v>15</v>
       </c>
-      <c r="I39">
+      <c r="I38">
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A40" s="4">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="4">
         <f>TIME(14,30,0)</f>
         <v>0.60416666666666663</v>
       </c>
+      <c r="B39" s="6">
+        <f>_xlfn.COT(A39)</f>
+        <v>1.4487060064955717</v>
+      </c>
+      <c r="C39" s="6">
+        <f>_xlfn.CSC(A39)</f>
+        <v>1.7603264166785513</v>
+      </c>
+      <c r="D39" s="6">
+        <f>_xlfn.SEC(A39)</f>
+        <v>1.2151025872646106</v>
+      </c>
+      <c r="E39" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B40" s="6">
-        <f>_xlfn.COT(A40)</f>
-        <v>1.4487060064955717</v>
-      </c>
-      <c r="C40" s="6">
-        <f>_xlfn.CSC(A40)</f>
-        <v>1.7603264166785513</v>
-      </c>
-      <c r="D40" s="6">
-        <f>_xlfn.SEC(A40)</f>
-        <v>1.2151025872646106</v>
-      </c>
-      <c r="E40" t="s">
-        <v>16</v>
-      </c>
-      <c r="I40">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B41" s="6">
         <f>_xlfn.COT(I:I)</f>
         <v>-0.29581291553274552</v>
       </c>
-      <c r="C41" s="6">
+      <c r="C40" s="6">
         <f>_xlfn.CSC(I:I)</f>
         <v>-1.0428352127714058</v>
       </c>
-      <c r="D41" s="6">
+      <c r="D40" s="6">
         <f>_xlfn.SEC(I:I)</f>
         <v>3.5253200858160887</v>
       </c>
+      <c r="E40" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <f>1.05*(0.0284+0.0046)-0.0284</f>
+        <v>6.2499999999999986E-3</v>
+      </c>
+      <c r="B41" s="6">
+        <f>_xlfn.COT(A41)</f>
+        <v>159.99791666124133</v>
+      </c>
+      <c r="C41" s="6">
+        <f>_xlfn.CSC(A41)</f>
+        <v>160.0010416714139</v>
+      </c>
+      <c r="D41" s="6">
+        <f>_xlfn.SEC(A41)</f>
+        <v>1.0000195315678966</v>
+      </c>
       <c r="E41" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I41">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42">
-        <f>1.05*(0.0284+0.0046)-0.0284</f>
-        <v>6.2499999999999986E-3</v>
+        <f>I43</f>
+        <v>1.75</v>
       </c>
       <c r="B42" s="6">
         <f>_xlfn.COT(A42)</f>
-        <v>159.99791666124133</v>
+        <v>-0.18114695257159807</v>
       </c>
       <c r="C42" s="6">
         <f>_xlfn.CSC(A42)</f>
-        <v>160.0010416714139</v>
+        <v>1.01627467666275</v>
       </c>
       <c r="D42" s="6">
         <f>_xlfn.SEC(A42)</f>
-        <v>1.0000195315678966</v>
+        <v>-5.6102223208037056</v>
       </c>
       <c r="E42" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I42">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43">
-        <f>I44</f>
+      <c r="A43" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="6" t="e">
+        <f>_xlfn.COT(A43)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C43" s="6" t="e">
+        <f>_xlfn.CSC(A43)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D43" s="6" t="e">
+        <f>_xlfn.SEC(A43)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I43">
         <v>1.75</v>
       </c>
-      <c r="B43" s="6">
-        <f>_xlfn.COT(A43)</f>
-        <v>-0.18114695257159807</v>
-      </c>
-      <c r="C43" s="6">
-        <f>_xlfn.CSC(A43)</f>
-        <v>1.01627467666275</v>
-      </c>
-      <c r="D43" s="6">
-        <f>_xlfn.SEC(A43)</f>
-        <v>-5.6102223208037056</v>
-      </c>
-      <c r="E43" t="s">
-        <v>19</v>
-      </c>
-      <c r="I43">
-        <v>7</v>
-      </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>20</v>
-      </c>
-      <c r="B44" s="6" t="e">
+      <c r="A44">
+        <f>PI() - 0.000000000001</f>
+        <v>3.141592653588793</v>
+      </c>
+      <c r="B44" s="7">
         <f>_xlfn.COT(A44)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C44" s="6" t="e">
+        <v>-999788629259.20374</v>
+      </c>
+      <c r="C44" s="7">
         <f>_xlfn.CSC(A44)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D44" s="6" t="e">
+        <v>999788629259.20374</v>
+      </c>
+      <c r="D44" s="6">
         <f>_xlfn.SEC(A44)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I44">
-        <v>1.75</v>
+        <v>-1</v>
+      </c>
+      <c r="E44" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45">
-        <f>PI() - 0.000000000001</f>
-        <v>3.141592653588793</v>
+        <f>PI()/2 - 0.000000000001</f>
+        <v>1.5707963267938965</v>
       </c>
       <c r="B45" s="7">
         <f>_xlfn.COT(A45)</f>
-        <v>-999788629259.20374</v>
-      </c>
-      <c r="C45" s="7">
+        <v>1.0001501580050864E-12</v>
+      </c>
+      <c r="C45" s="6">
         <f>_xlfn.CSC(A45)</f>
-        <v>999788629259.20374</v>
-      </c>
-      <c r="D45" s="6">
+        <v>1</v>
+      </c>
+      <c r="D45" s="7">
         <f>_xlfn.SEC(A45)</f>
-        <v>-1</v>
+        <v>999849864538.95483</v>
       </c>
       <c r="E45" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46">
-        <f>PI()/2 - 0.000000000001</f>
-        <v>1.5707963267938965</v>
+        <f>PI()/2 + 0.000000000001</f>
+        <v>1.5707963267958966</v>
       </c>
       <c r="B46" s="7">
         <f>_xlfn.COT(A46)</f>
-        <v>1.0001501580050864E-12</v>
+        <v>-1.0000276431595956E-12</v>
       </c>
       <c r="C46" s="6">
         <f>_xlfn.CSC(A46)</f>
@@ -5787,72 +5759,51 @@
       </c>
       <c r="D46" s="7">
         <f>_xlfn.SEC(A46)</f>
-        <v>999849864538.95483</v>
+        <v>-999972357604.52759</v>
       </c>
       <c r="E46" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A47">
-        <f>PI()/2 + 0.000000000001</f>
-        <v>1.5707963267958966</v>
-      </c>
-      <c r="B47" s="7">
+      <c r="A47" s="9">
+        <f>PI()/4</f>
+        <v>0.78539816339744828</v>
+      </c>
+      <c r="B47" s="6">
         <f>_xlfn.COT(A47)</f>
-        <v>-1.0000276431595956E-12</v>
+        <v>1</v>
       </c>
       <c r="C47" s="6">
         <f>_xlfn.CSC(A47)</f>
-        <v>1</v>
-      </c>
-      <c r="D47" s="7">
+        <v>1.4142135623730951</v>
+      </c>
+      <c r="D47" s="6">
         <f>_xlfn.SEC(A47)</f>
-        <v>-999972357604.52759</v>
+        <v>1.4142135623730949</v>
       </c>
       <c r="E47" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="10">
-        <f>PI()/4</f>
-        <v>0.78539816339744828</v>
+      <c r="A48" s="9">
+        <f>PI()/6</f>
+        <v>0.52359877559829882</v>
       </c>
       <c r="B48" s="6">
         <f>_xlfn.COT(A48)</f>
-        <v>1</v>
+        <v>1.7320508075688774</v>
       </c>
       <c r="C48" s="6">
         <f>_xlfn.CSC(A48)</f>
-        <v>1.4142135623730951</v>
+        <v>2</v>
       </c>
       <c r="D48" s="6">
         <f>_xlfn.SEC(A48)</f>
-        <v>1.4142135623730949</v>
+        <v>1.1547005383792515</v>
       </c>
       <c r="E48" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="10">
-        <f>PI()/6</f>
-        <v>0.52359877559829882</v>
-      </c>
-      <c r="B49" s="6">
-        <f>_xlfn.COT(A49)</f>
-        <v>1.7320508075688774</v>
-      </c>
-      <c r="C49" s="6">
-        <f>_xlfn.CSC(A49)</f>
-        <v>2</v>
-      </c>
-      <c r="D49" s="6">
-        <f>_xlfn.SEC(A49)</f>
-        <v>1.1547005383792515</v>
-      </c>
-      <c r="E49" t="s">
         <v>43</v>
       </c>
     </row>
@@ -6810,7 +6761,7 @@
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="10">
+      <c r="A48" s="9">
         <f>PI()</f>
         <v>3.1415926535897931</v>
       </c>
@@ -6831,7 +6782,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="10">
+      <c r="A49" s="9">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
@@ -6852,7 +6803,7 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="10">
+      <c r="A50" s="9">
         <f>2*PI()</f>
         <v>6.2831853071795862</v>
       </c>
@@ -6873,7 +6824,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="10">
+      <c r="A51" s="9">
         <f>PI()/4</f>
         <v>0.78539816339744828</v>
       </c>
@@ -6894,7 +6845,7 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="10">
+      <c r="A52" s="9">
         <f>PI()/6</f>
         <v>0.52359877559829882</v>
       </c>
@@ -6915,7 +6866,7 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="10">
+      <c r="A53" s="9">
         <v>10</v>
       </c>
       <c r="B53" s="6">
@@ -6932,7 +6883,7 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="10">
+      <c r="A54" s="9">
         <v>0.88</v>
       </c>
       <c r="B54" s="6">
@@ -6952,7 +6903,7 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" s="10">
+      <c r="A55" s="9">
         <v>0.44068679999999999</v>
       </c>
       <c r="B55" s="6">
@@ -7738,7 +7689,7 @@
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A48" s="10">
+      <c r="A48" s="9">
         <f>PI()</f>
         <v>3.1415926535897931</v>
       </c>
@@ -7755,7 +7706,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A49" s="10">
+      <c r="A49" s="9">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
@@ -7772,7 +7723,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" s="10">
+      <c r="A50" s="9">
         <f>2*PI()</f>
         <v>6.2831853071795862</v>
       </c>
@@ -7789,7 +7740,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" s="10">
+      <c r="A51" s="9">
         <f>PI()/4</f>
         <v>0.78539816339744828</v>
       </c>
@@ -7806,7 +7757,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" s="10">
+      <c r="A52" s="9">
         <f>PI()/6</f>
         <v>0.52359877559829882</v>
       </c>
@@ -7823,7 +7774,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A53" s="10">
+      <c r="A53" s="9">
         <v>10</v>
       </c>
       <c r="B53" s="6">

</xml_diff>